<commit_message>
all the fun updates
</commit_message>
<xml_diff>
--- a/TechComm/assignments/fact-sheet/fact_sheet_rubric_import_weighted.xlsx
+++ b/TechComm/assignments/fact-sheet/fact_sheet_rubric_import_weighted.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/85df9cffced7e2ed/Documents/github/tracigardner.github.io/TechComm/assignments/fact-sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2E6E061-2D40-4F15-88DB-2D3FB38FC97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="8_{C2E6E061-2D40-4F15-88DB-2D3FB38FC97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E57F249-BD49-425A-9072-7AF85A5D3549}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="195" windowWidth="19815" windowHeight="14895" xr2:uid="{557D898E-D278-48FA-902C-36654FEEB18F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{557D898E-D278-48FA-902C-36654FEEB18F}"/>
   </bookViews>
   <sheets>
     <sheet name="fact_sheet_rubric_import_weight" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="64">
   <si>
     <t>title_or_outcome_id</t>
   </si>
@@ -76,9 +89,6 @@
     <t>Rating_description_5</t>
   </si>
   <si>
-    <t>Pre-Check: Format &amp; Requirements</t>
-  </si>
-  <si>
     <t>Meets all basic format and assignment requirements: Exactly 1 page (front &amp; back); All required components present (title, intro, key facts, conclusion, visuals, sources); Minimum 3 visuals (incl. 1 data viz) ;Sources included and documented</t>
   </si>
   <si>
@@ -212,6 +222,9 @@
   </si>
   <si>
     <t>Hard to understand</t>
+  </si>
+  <si>
+    <t>The Basics: Minimum Requirements</t>
   </si>
 </sst>
 </file>
@@ -695,8 +708,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1072,391 +1088,437 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C417B9-99D4-4324-B568-98E62C289138}">
-  <dimension ref="A1:R8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S8"/>
+  <sheetFormatPr defaultColWidth="52.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="35.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="1" customWidth="1"/>
+    <col min="4" max="5" width="5" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="22.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="3.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="19.5703125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="4.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="19.140625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="6" style="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="16.85546875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.5703125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="16.5703125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="17.140625" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="52.28515625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <v>75</v>
+      </c>
+      <c r="E2" s="1">
+        <v>75</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C2" t="b">
+      <c r="J2" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="D2">
-        <v>75</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D3" s="1">
+        <v>30</v>
+      </c>
+      <c r="E3" s="1">
+        <v>3</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="1">
+        <v>26</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" s="1">
         <v>22</v>
       </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2">
+      <c r="L3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N3" s="1">
+        <v>19</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q3" s="1">
         <v>0</v>
       </c>
-      <c r="H2" t="s">
+      <c r="R3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="1">
+        <v>25</v>
+      </c>
+      <c r="E4" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="1">
+        <v>21</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="1">
+        <v>19</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" s="1">
+        <v>16</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>0</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1">
         <v>20</v>
       </c>
-      <c r="I2" t="s">
-        <v>21</v>
+      <c r="E5" s="1">
+        <v>2</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H5" s="1">
+        <v>17</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="K5" s="1">
+        <v>15</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="N5" s="1">
+        <v>13</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>0</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="6" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1">
+        <v>15</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C3" t="b">
+      <c r="G6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H6" s="1">
+        <v>13</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="K6" s="1">
+        <v>11</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N6" s="1">
+        <v>10</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q6" s="1">
         <v>0</v>
       </c>
-      <c r="D3">
-        <v>30</v>
-      </c>
-      <c r="E3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="R6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" s="1">
+        <v>10</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="1">
+        <v>8</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G3">
-        <v>26</v>
-      </c>
-      <c r="H3" t="s">
-        <v>28</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="J7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K7" s="1">
+        <v>7</v>
+      </c>
+      <c r="L7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J3">
-        <v>22</v>
-      </c>
-      <c r="K3" t="s">
-        <v>30</v>
-      </c>
-      <c r="L3" t="s">
+      <c r="M7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N7" s="1">
+        <v>6</v>
+      </c>
+      <c r="O7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M3">
-        <v>19</v>
-      </c>
-      <c r="N3" t="s">
-        <v>32</v>
-      </c>
-      <c r="O3" t="s">
+      <c r="P7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>0</v>
+      </c>
+      <c r="R7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>34</v>
-      </c>
-      <c r="R3" t="s">
-        <v>35</v>
+      <c r="S7" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>25</v>
-      </c>
-      <c r="E4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G4">
-        <v>21</v>
-      </c>
-      <c r="H4" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J4">
-        <v>19</v>
-      </c>
-      <c r="K4" t="s">
-        <v>30</v>
-      </c>
-      <c r="L4" t="s">
-        <v>40</v>
-      </c>
-      <c r="M4">
-        <v>16</v>
-      </c>
-      <c r="N4" t="s">
-        <v>32</v>
-      </c>
-      <c r="O4" t="s">
-        <v>41</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>34</v>
-      </c>
-      <c r="R4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>20</v>
-      </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5">
-        <v>17</v>
-      </c>
-      <c r="H5" t="s">
-        <v>28</v>
-      </c>
-      <c r="I5" t="s">
-        <v>46</v>
-      </c>
-      <c r="J5">
-        <v>15</v>
-      </c>
-      <c r="K5" t="s">
-        <v>30</v>
-      </c>
-      <c r="L5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M5">
-        <v>13</v>
-      </c>
-      <c r="N5" t="s">
-        <v>32</v>
-      </c>
-      <c r="O5" t="s">
-        <v>48</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>34</v>
-      </c>
-      <c r="R5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" t="b">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>15</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6">
-        <v>13</v>
-      </c>
-      <c r="H6" t="s">
-        <v>28</v>
-      </c>
-      <c r="I6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J6">
-        <v>11</v>
-      </c>
-      <c r="K6" t="s">
-        <v>30</v>
-      </c>
-      <c r="L6" t="s">
-        <v>54</v>
-      </c>
-      <c r="M6">
-        <v>10</v>
-      </c>
-      <c r="N6" t="s">
-        <v>32</v>
-      </c>
-      <c r="O6" t="s">
-        <v>55</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>34</v>
-      </c>
-      <c r="R6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>10</v>
-      </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G7">
-        <v>8</v>
-      </c>
-      <c r="H7" t="s">
-        <v>28</v>
-      </c>
-      <c r="I7" t="s">
-        <v>60</v>
-      </c>
-      <c r="J7">
-        <v>7</v>
-      </c>
-      <c r="K7" t="s">
-        <v>30</v>
-      </c>
-      <c r="L7" t="s">
-        <v>61</v>
-      </c>
-      <c r="M7">
-        <v>6</v>
-      </c>
-      <c r="N7" t="s">
-        <v>32</v>
-      </c>
-      <c r="O7" t="s">
-        <v>62</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>34</v>
-      </c>
-      <c r="R7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="D8">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="D8" s="1">
         <v>100</v>
       </c>
-      <c r="G8">
+      <c r="E8" s="1">
+        <f>SUM(E2:E7)</f>
         <v>85</v>
       </c>
-      <c r="J8">
-        <f>SUM(J3:J7)</f>
+      <c r="H8" s="1">
+        <v>85</v>
+      </c>
+      <c r="K8" s="1">
+        <f>SUM(K3:K7)</f>
         <v>74</v>
       </c>
-      <c r="M8">
-        <f>SUM(M3:M7)</f>
+      <c r="N8" s="1">
+        <f>SUM(N3:N7)</f>
         <v>64</v>
       </c>
-      <c r="P8">
-        <f>SUM(P3:P7)</f>
+      <c r="Q8" s="1">
+        <f>SUM(Q3:Q7)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
creating rubric and self-check
</commit_message>
<xml_diff>
--- a/TechComm/assignments/fact-sheet/fact_sheet_rubric_import_weighted.xlsx
+++ b/TechComm/assignments/fact-sheet/fact_sheet_rubric_import_weighted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/85df9cffced7e2ed/Documents/github/tracigardner.github.io/TechComm/assignments/fact-sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{C2E6E061-2D40-4F15-88DB-2D3FB38FC97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E57F249-BD49-425A-9072-7AF85A5D3549}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="8_{C2E6E061-2D40-4F15-88DB-2D3FB38FC97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03D1CD6A-AD1A-4939-8748-F801A01F76FF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{557D898E-D278-48FA-902C-36654FEEB18F}"/>
+    <workbookView xWindow="1815" yWindow="0" windowWidth="25395" windowHeight="14895" xr2:uid="{557D898E-D278-48FA-902C-36654FEEB18F}"/>
   </bookViews>
   <sheets>
     <sheet name="fact_sheet_rubric_import_weight" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
   <si>
     <t>title_or_outcome_id</t>
   </si>
@@ -1088,31 +1088,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C417B9-99D4-4324-B568-98E62C289138}">
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr defaultColWidth="52.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="35.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="11.42578125" style="1" customWidth="1"/>
-    <col min="4" max="5" width="5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="22.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="3.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="19.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="4.42578125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="19.140625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="6" style="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="16.85546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="3.5703125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="17.140625" style="1" customWidth="1"/>
-    <col min="20" max="16384" width="52.28515625" style="1"/>
+    <col min="4" max="4" width="5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="4.42578125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="19.140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="6" style="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="16.85546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="3.5703125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="16.5703125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="17.140625" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="52.28515625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1126,52 +1126,49 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>63</v>
       </c>
@@ -1184,26 +1181,23 @@
       <c r="D2" s="1">
         <v>75</v>
       </c>
-      <c r="E2" s="1">
-        <v>75</v>
+      <c r="E2" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="1">
+      <c r="G2" s="1">
         <v>0</v>
       </c>
+      <c r="H2" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="I2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>23</v>
       </c>
@@ -1216,53 +1210,50 @@
       <c r="D3" s="1">
         <v>30</v>
       </c>
-      <c r="E3" s="1">
-        <v>3</v>
+      <c r="E3" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="1">
+      <c r="G3" s="1">
         <v>26</v>
       </c>
+      <c r="H3" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="1">
+      <c r="J3" s="1">
         <v>22</v>
       </c>
+      <c r="K3" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="L3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N3" s="1">
+      <c r="M3" s="1">
         <v>19</v>
       </c>
+      <c r="N3" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="O3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="P3" s="1">
         <v>0</v>
       </c>
+      <c r="Q3" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="R3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="S3" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -1275,53 +1266,50 @@
       <c r="D4" s="1">
         <v>25</v>
       </c>
-      <c r="E4" s="1">
-        <v>2.5</v>
+      <c r="E4" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="1">
+      <c r="G4" s="1">
         <v>21</v>
       </c>
+      <c r="H4" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="K4" s="1">
+      <c r="J4" s="1">
         <v>19</v>
       </c>
+      <c r="K4" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="L4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="M4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="N4" s="1">
+      <c r="M4" s="1">
         <v>16</v>
       </c>
+      <c r="N4" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="O4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="P4" s="1">
         <v>0</v>
       </c>
+      <c r="Q4" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="R4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="S4" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>42</v>
       </c>
@@ -1334,53 +1322,50 @@
       <c r="D5" s="1">
         <v>20</v>
       </c>
-      <c r="E5" s="1">
-        <v>2</v>
+      <c r="E5" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="1">
+      <c r="G5" s="1">
         <v>17</v>
       </c>
+      <c r="H5" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K5" s="1">
+      <c r="J5" s="1">
         <v>15</v>
       </c>
+      <c r="K5" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="L5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="M5" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="N5" s="1">
+      <c r="M5" s="1">
         <v>13</v>
       </c>
+      <c r="N5" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="O5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="P5" s="1">
         <v>0</v>
       </c>
+      <c r="Q5" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="R5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="S5" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>49</v>
       </c>
@@ -1393,53 +1378,50 @@
       <c r="D6" s="1">
         <v>15</v>
       </c>
-      <c r="E6" s="1">
-        <v>1.5</v>
+      <c r="E6" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="H6" s="1">
+      <c r="G6" s="1">
         <v>13</v>
       </c>
+      <c r="H6" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="K6" s="1">
+      <c r="J6" s="1">
         <v>11</v>
       </c>
+      <c r="K6" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="L6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="M6" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N6" s="1">
+      <c r="M6" s="1">
         <v>10</v>
       </c>
+      <c r="N6" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="O6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P6" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="P6" s="1">
         <v>0</v>
       </c>
+      <c r="Q6" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="R6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="S6" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>56</v>
       </c>
@@ -1452,73 +1434,66 @@
       <c r="D7" s="1">
         <v>10</v>
       </c>
-      <c r="E7" s="1">
-        <v>1</v>
+      <c r="E7" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="1">
+      <c r="G7" s="1">
         <v>8</v>
       </c>
+      <c r="H7" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K7" s="1">
+      <c r="J7" s="1">
         <v>7</v>
       </c>
+      <c r="K7" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="L7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="M7" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N7" s="1">
+      <c r="M7" s="1">
         <v>6</v>
       </c>
+      <c r="N7" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="O7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P7" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="P7" s="1">
         <v>0</v>
       </c>
+      <c r="Q7" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="R7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="S7" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="D8" s="1">
         <v>100</v>
       </c>
-      <c r="E8" s="1">
-        <f>SUM(E2:E7)</f>
+      <c r="G8" s="1">
         <v>85</v>
       </c>
-      <c r="H8" s="1">
-        <v>85</v>
-      </c>
-      <c r="K8" s="1">
-        <f>SUM(K3:K7)</f>
+      <c r="J8" s="1">
+        <f>SUM(J3:J7)</f>
         <v>74</v>
       </c>
-      <c r="N8" s="1">
-        <f>SUM(N3:N7)</f>
+      <c r="M8" s="1">
+        <f>SUM(M3:M7)</f>
         <v>64</v>
       </c>
-      <c r="Q8" s="1">
-        <f>SUM(Q3:Q7)</f>
+      <c r="P8" s="1">
+        <f>SUM(P3:P7)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>